<commit_message>
Cursor session analysis artifacts
</commit_message>
<xml_diff>
--- a/KT_Session_Question_Analysis/SHRSS_Adobe_KT_Session_Follow_Up_Tracker.xlsx
+++ b/KT_Session_Question_Analysis/SHRSS_Adobe_KT_Session_Follow_Up_Tracker.xlsx
@@ -455,6 +455,9 @@
   </sheetPr>
   <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="84.83203125" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="1" s="2">
       <c r="A1" s="1" t="inlineStr">
@@ -576,7 +579,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -656,7 +658,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -694,7 +695,6 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -732,7 +732,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -770,7 +769,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -808,7 +806,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -846,7 +843,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -926,7 +922,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1006,7 +1001,6 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1044,7 +1038,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1124,7 +1117,6 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1162,7 +1154,6 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1284,7 +1275,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1322,7 +1312,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1444,7 +1433,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1482,7 +1470,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1562,7 +1549,6 @@
           <t>Deferred</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1600,7 +1586,6 @@
           <t>Deferred</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1680,7 +1665,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1844,7 +1828,6 @@
           <t>Answered</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1882,7 +1865,6 @@
           <t>Deferred</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1920,7 +1902,6 @@
           <t>Deferred</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2042,7 +2023,6 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2080,7 +2060,6 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2118,7 +2097,6 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2156,7 +2134,6 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2179,8 +2156,6 @@
           <t>Not answered in session. Initial setup by Adobe; full list and process to be confirmed (Vinay, IT).</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>Pending</t>
@@ -2213,8 +2188,6 @@
           <t>Not answered in session.</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>Pending</t>
@@ -2247,8 +2220,6 @@
           <t>Not answered in session. Categories from Workday; author-created jobs must match exact category string.</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>Pending</t>
@@ -2281,8 +2252,6 @@
           <t>Not explicitly listed in session. Many items taken as follow-up or gap analysis.</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>Pending</t>
@@ -2315,8 +2284,6 @@
           <t>Not answered in session.</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>Pending</t>
@@ -2339,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="24.83203125" customWidth="1" min="1" max="1"/>
@@ -2385,6 +2352,1077 @@
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>View as published shows changes fast but publisher takes too long; new job (CF) not showing on publisher. Can we expedite?</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Gonzalo Calasich (SHRSS)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Need more info (cache, etc.). Daniela will monitor during call. Andy investigating failed publish logs; will raise support ticket.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Daniela Tea / Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Gonzalo: not showing at all on publisher; likely cache.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Override for date field (e.g. 'every Wednesday through February') instead of actual date/time?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Not in event content fragment. Promotions has date override; can confirm if same behavior wanted for events—gap.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Same question for location override.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>What happens if we add an additional image in the event image field (multi)?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Believes it defaults to first one; can test. Migration used only one image.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Event status: logic so presale dates show presale disclaimer then auto-revert to 'on sale'?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Not currently. Gap: associate status with date/time so it changes without author republish. Presale can be outside business hours.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hide CTA (more info) when there's no landing page / no extra info for user?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Default links to event detail page. Toggle to hide CTA entirely would be gap.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Use case: weekly free entertainment; no detail page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Location reference: limit by user so cafe only adds their location? Avoid choosing wrong location (e.g. Amsterdam for Mexico event).</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Location reference drives filter roll-up; root path limits which events show. Wrong location in CF still adds to this site's filter. Restrict by user = gap.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Folder path = organization; location reference = required for display/filter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Default image for event card so author doesn't have to select every time (generic default)?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CF cannot be saved without image. Component-level default (like jobs listing) could be gap. Author can use default from DAM in meantime.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Event detail page—why does it look like a card? Are we on careers? Hard Rock Live—can we use for careers?</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>This is the event detail page (one template). Same for all sites. Daniela created new page to show from scratch.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Mayte: digital page not working for careers events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Clean/friendly URL for event detail (property.com/artist-name not numbers)?</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Lisa Cardia / Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Event ID is read-only to prevent duplicates. Enhancement = make editable for friendly URL. Mayte: need real names; like WordPress/Sitecore—pick up page name. Gap.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Labor intensive; add to gap list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Event detail page hero—standard across all or customizable per page?</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Default hero on event detail page; banner image + alt in CF overrides.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Event statuses: all manual or can we schedule (presale, announcement, rescheduled)? Do they drive/hide content?</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Currently manual. Gap to have date range per status. Presale/sold out etc. change label/flag; event status message is separate. Doesn't hide CTA or content.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Do we have to publish to see changes? How to preview before publish for approval?</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lisa Cardia / Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>View as published doesn't show CF changes until CF is published. Andy: preview tier exists, not configured; will check export. Mayte: need browser preview to screenshot for approval.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Daniela Tea / Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Preview server / preview links = gap analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>When adding new event: publish fragment, detail page, and calendar every time?</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>One event detail page per calendar—publish once. New event: publish CF; calendar page must be published for event to show on publisher (can take a few minutes).</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Gonzalo's delay = calendar page publish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Unpublish event (take down without delete) to repurpose later?</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lisa Cardia / Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Unpublish CF removes from calendar. Daniela to check if detail URL still accessible. Later: unpublished = detail URL shows configured 'no events' message; content not visible.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Mayte: add as gap—not expected behavior but at least user doesn't see it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Recap: unpublish works; schedule not local to property; end date auto drop-off; all statuses manual; no date/location override; three times instead of one (vs Sitecore).</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Daniela acknowledged. Hiring events use promotions model (has overrides); events model does not.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Mayte Eme / Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Hiring events—using promotions not events? What can events CF do vs promotions?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mayte Eme / Gonzalo</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Hiring events section uses promotions content fragment (date/location override). Events CF + calendar/detail = what we covered. Tomorrow: hiring events component.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Careers not using events CF for that section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Can we choose mix-and-match locations for one calendar (e.g. six properties, or hotel+casinos, or by venue)?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>No. One content fragment folder path only; cannot select multiple folders. Big gap for multi-venue/entertainment sites.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Pull events into other pages (venue page, homepage by category, e.g. dinner and a show)?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Content Fragment card list component can show events (or news); by root path or by tag (e.g. dinner and a show). Not locked to calendar component.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Why did we lose the filter for events (careers hiring events landing page)?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Careers uses content fragment card (no filter on purpose for homepage). Promotions component has filter; can swap on landing page if desired.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Can we pull jobs (hot jobs/hiring events) to property page (e.g. Reverb) by tag or location?</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Yes—select root path (e.g. Tampa folder); all jobs under that path. Cannot select multiple locations in one component. Exclude category under Tampa? Not in component.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Display tag on event cards (21+, free event, phone-free)?</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Daniela asked for example; will discuss with technical team.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Edwin to send example.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Preview link for unpublished page to share for approval before republish?</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Rick Lyon (Director of Digital Experience)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Unpublished CF not on calendar or detail. If publish CF, visible in author; page must be published for end user. Daniela to report back on detail-page behavior.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Preview before publish = gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Publish delays on stage—investigating?</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Lucas Nelson</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Andy: seen failed publish entries in cloud services log; raising support ticket; will keep team posted.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Governance: Who owns Event Categories tags and DPLT location list? Process when property/venue added or renamed?</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Authoring: One-page checklist for event authoring (what to create, publish, order) and when to use events CF vs promotions CF?</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tagging: Event categories vs tags for filtering vs 'dinner and a show' query—who governs?</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Not answered in session. Categories = filter; tags = internal; tag for query possible.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Gap analysis: Decision criteria for events CF vs promotions CF; which gaps apply to which model?</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Permissions: Who can create/edit Event Categories tags and DPLT location reference options?</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
         </is>
       </c>
     </row>
@@ -2399,7 +3437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -2451,6 +3489,1242 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Manual job content fragment: create, publish, not showing on jobs page. Other CFs show. Workday sync deletes manual jobs (is not API data) in ~30 min.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Gonzalo Calasich (SHRSS)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Andy: investigating; support ticket. Get all job IDs not excluding manual; email with recommendation coming; tech sync to drill in.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Andy Lambert / Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Gonzalo to send example URLs for logs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Promotion ID—where from? What do we put? Is it made up? Required for targeting/analytics we had for casino, not unique ID for display.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lisa Cardia / Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Author-entered unique identifier to display one promotion (e.g. content fragment card). No format requirement. Uniqueness validated on save. Same value in another CF blocks save.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Mayte: gap—we don't want this; need to remember/copy; not smart (dropdown of existing IDs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>When pasting ID elsewhere (e.g. component), is there a dropdown to select from existing or must we remember/paste?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Component field is plain text; no dropdown. Must copy from CF. Gonzalo: gap = source field to navigate DAM and pick CF.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Without promotions filter (careers homepage): steps to get card on page = know ID, copy from fragment, paste in component. No other way?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Yes. Content fragment card expects promotion ID for promotions/events. No folder path picker. Gap: enhance card list to include promotions or add path/source picker.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Promotion ID for casino or careers? We're not using for casinos; we need to fix for casinos (many users, can't remember IDs).</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Initially for casinos. Careers using it for hiring events. Lucas: capture what it doesn't have; disposition in platform expansion; modify/change is part of it.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Daniela Tea / Lucas Nelson</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Promotion search: can we remove the search field and keep only filters?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Search cannot be removed currently. With filters, search bar always shows. To display as list without filter/search = gap.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>If we use promotions for hiring events we can't have promotion cards in grid/carousel elsewhere without filter+search—only one-by-one by ID.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Correct. Content fragment card list currently events/news only; gap = add promotions so list/carousel without filter+search.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Who manages filter options (category, venue, date range)? Author or dev? Can we add different options?</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>In component code; hardcoded from promotions requirements. New filter = dev. Potential to move to generic list (author-managed) but not available today. Mayte: we manage every filter—gap.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Promotion search: same as events—can't select two category folders (e.g. casino + hotel promotions)?</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Single path only. Can choose promotions root or e.g. casinos; cannot pick two of four folders. Mayte: another gap.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Promotions: are filter options (e.g. select category) translatable / overridable for language?</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Daniela to check with tech team. Components have language strings; need to confirm what's translatable. At minimum override all areas. Gonzalo: include Transperfect + developer labels.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Technical topic; Scott/technical enablement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Transperfect: manual translations for some languages; not always Transperfect. OK?</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Noted. Daniela will address in Transperfect KT.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Promotion start/end date and time—is that for scheduling or display only?</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Display only. Schedule = Manage Publication &gt; Now or Later (activation date). Not for 'display this event on Saturday but publish tomorrow.'</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>If we schedule for later and then edit the fragment (e.g. change venue), does it maintain schedule or push live?</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Daniela to test (save, manage publication, save); will confirm.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Promo types (loyalty, slot)—hardcoded? How do we add extra promo types?</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>In content fragment model (not component). Model editor = more flexibility; permissions apply. Adding dropdown to component = dev. Model edit vs component = different.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Card/promotion image: 16:9 asset—how to control focal point (e.g. center guitar)? Image position?</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Image position tab on image components (desktop/tablet/mobile). List (promotion search) has no per-row position; crop outside or use rendition—DAM/gap.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Don: one source image across placements; figure out with DAM/renditions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Job listings on another site (e.g. hotel)—same component, theme changes styling? Can we choose multiple locations?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Yes—component is global; theme drives look. Still one root path only (gap). Use case: Tampa/Hollywood dedicated job pages.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>How do we see the promotion card's detail page? Is there a promotion detail template?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>No promotion detail template. Create open page, add content, link from CF. Daniela to show casino example from integration env.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Banner image in CF = for when promotion has its own page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Events template allows link to another page (event detail). Promotions can't do that—we have hot jobs/dealer university with detail pages.</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Promotions: can link to any page from CF. Events: one detail page + ID. Override in events = gap; then could use events for hiring events. Workaround: link to existing page from promotion CF.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Video card: external URL—recommended width? Pixel required? What does width affect?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Width affects modal size. Number only, no 'px.' 846 was to match live site. Can change.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Video card: third party (YouTube) gives fixed/responsive, aspect ratio; external URL doesn't. Same config for external?</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Lisa Cardia / Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>External URL = no those options. Third party = full config. Gap—external should have same controls; else only use YouTube/Vimeo. Mayte: don't use external until fixed.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Video card styling (none/black/white): is 'none' transparent? White description not showing.</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Daniela to check white; none = default. Black works. Screenshot of three when fixed.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Video card: if we add a fourth, does it become carousel automatically (like Sitecore)?</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>No. Video card not in allowed components for card carousel or hero carousel. Gap: allow video cards in carousel.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Card (icon variation): with 6 or 9 cards, does it go 3 to 1 columns automatically or manual per breakpoint?</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Manual per viewport for standalone card. Some components (e.g. carousel) have breakpoint config. Mayte: add to gap list.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Executives/diversity page (careers) same as hardrock.com—shared so one update?</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Currently separate cards. Can move to experience fragment: update once, same styling both sites. Content fragment = same content, different styling per site.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Rick: corporate page hardrock.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Experience fragment: same content, different styling per site possible?</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Experience fragment = same content + same look. For same content, different look = content fragment.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Asset specs for video card thumbnail, promotion card/banner—recommended dimensions? Focal point for video thumbnail?</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Document on component basis; video thumbnail aspect/specs; no image tab on video card. Gap.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Store component on page but not displayed (like Sitecore disable)—reuse later without recreating? Hide = still in DOM?</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Lisa Cardia / Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Hide component (layout &gt; eye) = still in tree, still in DOM/crawled. Not like Sitecore where disabled = not in HTML. Gap: store without rendering for evergreen swap.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Content refresh initiative; rotate temp vs evergreen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Careers locations page same as brand—pulling from DPLT? Can we copy accordion/component so one source?</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Careers = accordion/text (migrated); brand = map component + DPLT. Can copy map component to careers. Intent: all location listings from DPLT, one maintenance.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Daniela to post test page with copied component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Governance: Who owns promotion ID list and filter options? Process to add/change?</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Authoring: Single checklist for hiring events (CF → card vs search → detail page → publish order) and when events vs promotions?</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Tagging: Do promotions use tags for filtering? If card list adds promotions, tag-based selection?</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Gap priorities: Which items (ID vs path, filter removal, card list promotions, video carousel, thumbnail specs, hide vs disable) for careers vs platform expansion?</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Permissions: Who can edit promotions model (promo types) and promotion search config (filter labels)?</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2462,7 +4736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" customFormat="1" s="2">
@@ -2504,6 +4778,344 @@
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Why multiple category directories (categories, category, news categories, events categories)? Consolidate under one?</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Different purposes; naming could be clearer. Andy to assess functional implications of consolidation, then green-light. Add as to-do for cleanup.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Don: same for property/hotel/casino/cafe under locations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>If we restructure tags, does that break anything currently?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Assess first; goal is no hard-coded paths, config where possible. Then SHRSS can make changes. Move tool updates reference paths.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>How do we use generic lists (ACS Commons path-to-tag mapping)? What are they used for?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Governs tags for a section. Andy to add to Confluence Q&amp;A; Vinay for deeper answer. Not used for corporate/careers today.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Content fragment model category field—tag-driven or defined in model? Where do these lists come from?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Can be tag-driven or enumeration. Locations example = not all from tags. Depends on use case; gap to align. Check model.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Asset categories vs content fragment categories—different? Event categories on asset vs events.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Yes—asset metadata vs CF categories; confusing. Asset event categories ≠ CF event categories. Action: cleanup, rename for clarity.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Lisa: location reference ID same issue (events session).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pre-populated metadata set for export (so we don't add 15 properties every time)?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Not OOTB. Andy: pain; keep text file with property names, copy/paste. Chris may say same tomorrow.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Governance: Who owns SHRSS tag vocabulary and consolidation decision? Process to add namespace?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Authoring: Where do authors see tag-driven vs fixed list? One-pager by model/asset type?</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Permissions: Which groups have create/update/delete on SHRSS tags?</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Not answered in session. Andy: use groups; lock down.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
         </is>
       </c>
     </row>
@@ -2518,7 +5130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" customFormat="1" s="2">
@@ -2560,6 +5172,268 @@
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SHRSS primary: consolidate into SHRSS, deprecate primary? Path forward.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Yes. Don to move primary content into SHRSS; deprecate primary. Content fragment behavior may need back-end look.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Don: 13 months ago didn't know move wouldn't break refs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Legacy/migrated assets folder—option to move old content there, new structure for new?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Yes—e.g. legacy-assets; new content in new structure; cleanup/scripting later. Chris agreed.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Andy Lambert / Chris Lewis</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Language folders for assets—required for translation automation?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Chris: language at top level for AM Guide etc. If no language-swap use case, metadata for language is fine. Don: single asset, metadata.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Chris Lewis</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Renditions: Don tried to create, they're not applying.</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Andy: renditions in agenda; will cover. Hot topic.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Andy Lambert</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Careers asset names odd (C2D5 etc.)—not from Sitecore. Bulk rename?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Lisa Cardia / Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Chris: migration tool internal ref. Bulk rename via export metadata to Excel, edit names, re-upload.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Chris Lewis</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Governance: Who approves DAM folder structure and bulk renames?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rendition profiles not applying—root cause and fix in scope?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
         </is>
       </c>
     </row>
@@ -2574,7 +5448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" customFormat="1" s="2">
@@ -2616,6 +5490,230 @@
       <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Redirect vanity URL checkbox—what does it do? When to use?</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Daniela to get back. In this case not needed.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Multiple vanity URLs per page—all link to same page?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rick Lyon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Yes. Useful for print (short URL) vs long.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Card carousel tablet field removed—why? Can we have tablet-specific again?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Daniela Tea (update)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Requirement: desktop/tablet same, mobile separate. Tablet always 2 for non–full width; field had no effect. Removed. Gap if tablet config needed.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Content fragment model: default image for new CF? Override by author?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Yes—default value on model; new CFs get it; author can replace. Custom component (e.g. card) would show it.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Experience fragment variation: break connection to reorder or use as regular component?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Daniela to confirm.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Governance: Who creates CF models for shared data? Who creates EF variations and rolls out?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
         </is>
       </c>
     </row>
@@ -2630,7 +5728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -2682,6 +5780,268 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>List component: exclude certain tags (e.g. do not use) from list?</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Not OOTB; matching only. Daniela to take use case back (e.g. promotion page not on landing).</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>List: what dictates which items appear in which column? Order?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Order by title or last modified. Column count in config; fills in order.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Logo styling (image icon in footer)—what is it? Use case?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Daniela to check JIRA; not footer-specific; image component in general (e.g. height/width for multi-logo pages).</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Redirect vanity URL checkbox: 302 redirect; when to use?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Daniela Tea (update)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Documentation: 302 when checkbox. Daniela to share link; technical enablement for redirect management.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>News: default image by category/tag (e.g. casino vs hotel)?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Edwin Aquino</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Not currently. Gap; need requirements (multiple tags = which default?).</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>News CF: default image in model? Carlos: all articles have image.</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Carlos Aldana</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Default image at component level (news search results) for items without image. Model default can be added.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Governance: Who can add news categories (tags) and change news CF model?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2693,7 +6053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" customFormat="1" s="2">
@@ -2738,6 +6098,352 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Location CF title = location ID; how to bulk update to property legal name?</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Don Middlebrook</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bulk metadata update: take value from property legal name (or chosen field), replace title. Daniela: tech KT if help needed.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Read-only fields from DPLT; title editable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>New location from DPLT: is delivery only—author manually checks?</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Yes.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Image in location CF—where does it populate? Hotels?</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Destinations and venues component (e.g. Hard Rock Hotel Cancun). Image specs to Confluence.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Delivery/venue links: open in new window?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rick Lyon</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Yes; baked in (external links).</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Add new sort-by or filter field (e.g. meeting room view)? Process?</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Update venue CF model, add to component dialog, front-end component update. Mayte: gap—overcomplicated; need optimized way. Lucas: mark as gap.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Filters (e.g. type of destination) also hard-coded? Can we add (e.g. Unity participating hotel)?</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Lisa Cardia</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Same concept—model + component.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Regions filter on hardrock.com prod not working—Google Map component?</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Gonzalo Calasich (SHRSS)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Different component (Google Map). Destination search and filter = this one. Cover Google Map when we get to it.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Daniela Tea</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gap list: Adobe building it or SHRSS? Confluence questions = gap list?</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lisa Cardia / Mayte Eme</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Lucas: SHRSS documents gaps; Confluence questions feed funnel. Adobe shows framework; SHRSS comes to platform expansion with use cases and gaps.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Lucas Nelson</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Scott: questions/needs on Confluence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Governance: Who maintains location/venue CF when DPLT updates? Who can add new sort/filter fields?</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Product Director</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Not answered in session.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Product Director persona.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Locations, Day 2 and Media questions analysis
</commit_message>
<xml_diff>
--- a/KT_Session_Question_Analysis/SHRSS_Adobe_KT_Session_Follow_Up_Tracker.xlsx
+++ b/KT_Session_Question_Analysis/SHRSS_Adobe_KT_Session_Follow_Up_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lambert/Documents/Projects/SHRSS/SHRSS_Knowledge_Transfer/KT_Session_Question_Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F61CC25-0FD6-6A4E-B6D0-FA315C2E71BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31714BB1-897F-6B42-B3A0-B1F12F2B0D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jobs" sheetId="1" r:id="rId1"/>
@@ -21,13 +21,15 @@
     <sheet name="Shared_Data" sheetId="6" r:id="rId6"/>
     <sheet name="News" sheetId="7" r:id="rId7"/>
     <sheet name="Locations" sheetId="8" r:id="rId8"/>
+    <sheet name="Locations_Day_2" sheetId="9" r:id="rId9"/>
+    <sheet name="Media" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1302" uniqueCount="416">
   <si>
     <t>Status</t>
   </si>
@@ -1131,6 +1133,150 @@
   </si>
   <si>
     <t>Governance: Who maintains location/venue CF when DPLT updates? Who can add new sort/filter fields?</t>
+  </si>
+  <si>
+    <t>2026-02-24</t>
+  </si>
+  <si>
+    <t>What path do we choose for CF list path (category listing)? Not intuitive; can we update info tools?</t>
+  </si>
+  <si>
+    <t>Path = parent; component shows children of that parent. E.g. path to EN under news → year folders. Daniela demonstrated; Edwin confirmed.</t>
+  </si>
+  <si>
+    <t>News session follow-up.</t>
+  </si>
+  <si>
+    <t>Kerry Holyoak (SHRSS) / Daniela Tea</t>
+  </si>
+  <si>
+    <t>Delivery widget: Hard Rock Casino Rockford showing—casino classified as cafe. Who do we contact to fix?</t>
+  </si>
+  <si>
+    <t>DPLT team (Vipul Patel). Classifications come from DPLT; if misclassified, take to Vipul's team. Lisa to reach out.</t>
+  </si>
+  <si>
+    <t>Line of business = Cafe in DPLT drives delivery list.</t>
+  </si>
+  <si>
+    <t>Booking modal: black border; can we make booking widget same size/background as modal?</t>
+  </si>
+  <si>
+    <t>Note as gap—configurable color/size for modal.</t>
+  </si>
+  <si>
+    <t>Rick Lyon / Daniela Tea</t>
+  </si>
+  <si>
+    <t>Where do we get destination value (e.g. 59391) for booking widget? Do authors need to know it?</t>
+  </si>
+  <si>
+    <t>Rick: Senex/Vizergy; in booking links. Migrated; values don't change. Authors may need for restore if someone changes. Daniela: casino booking not finalized (pre-pause).</t>
+  </si>
+  <si>
+    <t>Booking widget: adding a different field (e.g. balcony) beyond rooms/adults/children—development?</t>
+  </si>
+  <si>
+    <t>Yes—new field type, UI, parameter passing, booking engine side. Development for sure.</t>
+  </si>
+  <si>
+    <t>Booking offers: can we hide the booking window section completely?</t>
+  </si>
+  <si>
+    <t>Tried; window still present, fields blank. Hide label too = potential gap. No option to hide completely today.</t>
+  </si>
+  <si>
+    <t>Find a location: can we change the background color?</t>
+  </si>
+  <si>
+    <t>Currently fixed in code. Change would require code update to allow author-configurable background.</t>
+  </si>
+  <si>
+    <t>Google Map: regions dropdown blank in prod—why? North America first in config but showing last.</t>
+  </si>
+  <si>
+    <t>Permissions: groups didn't have read on generic list 'regions.' Template Authors given read. Order: ensure regions authored in dialog (first = top); republish page.</t>
+  </si>
+  <si>
+    <t>ACS Commons on prod. Media session confirmed fix.</t>
+  </si>
+  <si>
+    <t>Google Map: filter map not in config but filters showing—why? No results vs no locations?</t>
+  </si>
+  <si>
+    <t>Filter map adds filters on map. Different messages for no results vs no locations. Daniela made copy to demo filter map.</t>
+  </si>
+  <si>
+    <t>Lisa Cardia / Rick Lyon</t>
+  </si>
+  <si>
+    <t>Google Map: carousel dots not centered under images.</t>
+  </si>
+  <si>
+    <t>Daniela noted; would need to be updated to center align carousel dots.</t>
+  </si>
+  <si>
+    <t>Who owns DPLT classification (line of business) and SHRSS contact for misclassification?</t>
+  </si>
+  <si>
+    <t>Which groups need read/write on generic list 'regions' for Google Map?</t>
+  </si>
+  <si>
+    <t>Not answered in session. Andy covering permissions in KT next week.</t>
+  </si>
+  <si>
+    <t>2026-02-25</t>
+  </si>
+  <si>
+    <t>Google Map regions dropdown not visible yesterday—resolution?</t>
+  </si>
+  <si>
+    <t>Generic list 'regions' populates dropdown. User groups lacked read access. Template Authors given read; Gonzalo and Lisa confirmed can see. Permissions topic with Andy next week.</t>
+  </si>
+  <si>
+    <t>Locations Day 2 follow-up.</t>
+  </si>
+  <si>
+    <t>North America showing last on prod—publish page again?</t>
+  </si>
+  <si>
+    <t>View as published to confirm order; then publish. Andy to take a look at prod page.</t>
+  </si>
+  <si>
+    <t>Media gallery: carousel dots not centered (left of center).</t>
+  </si>
+  <si>
+    <t>Daniela noted; capture for update to center align carousel dots.</t>
+  </si>
+  <si>
+    <t>Image gallery grid: option to show/hide title or inherit from asset like alt text?</t>
+  </si>
+  <si>
+    <t>Not for this component. Title pulled from DAM metadata. If no title in metadata, 'no title' shows. Enhancement to capture if team wants option to not display title.</t>
+  </si>
+  <si>
+    <t>Image gallery grid: different titles for same image per property/site?</t>
+  </si>
+  <si>
+    <t>Not currently. Control via metadata per asset; no variation/title override in component.</t>
+  </si>
+  <si>
+    <t>Don Middlebrook / Daniela Tea</t>
+  </si>
+  <si>
+    <t>Daniela Tea (to Don)</t>
+  </si>
+  <si>
+    <t>Image gallery grid: are we adding titles/descriptions to assets?</t>
+  </si>
+  <si>
+    <t>Don: planning to add as much metadata as possible—titles, description. Daniela: if titles not always desired, capture enhancement to not display or use description.</t>
+  </si>
+  <si>
+    <t>Who can add/edit generic list values (e.g. regions)? Which groups get read vs write?</t>
+  </si>
+  <si>
+    <t>Image gallery grid: hide title or show description—enhancement?</t>
   </si>
 </sst>
 </file>
@@ -1514,7 +1660,9 @@
     <col min="2" max="2" width="15.6640625" customWidth="1"/>
     <col min="3" max="3" width="17.1640625" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" customWidth="1"/>
+    <col min="6" max="6" width="62.83203125" customWidth="1"/>
+    <col min="7" max="7" width="41.33203125" customWidth="1"/>
     <col min="8" max="8" width="67.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2687,6 +2835,230 @@
       <c r="H48" t="s">
         <v>137</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" customWidth="1"/>
+    <col min="4" max="4" width="25.5" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" customWidth="1"/>
+    <col min="6" max="6" width="55" customWidth="1"/>
+    <col min="7" max="7" width="51.33203125" customWidth="1"/>
+    <col min="8" max="8" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>398</v>
+      </c>
+      <c r="C2" t="s">
+        <v>398</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>398</v>
+      </c>
+      <c r="C3" t="s">
+        <v>398</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>398</v>
+      </c>
+      <c r="C4" t="s">
+        <v>398</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>322</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" t="s">
+        <v>398</v>
+      </c>
+      <c r="C5" t="s">
+        <v>398</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>165</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
+        <v>398</v>
+      </c>
+      <c r="C6" t="s">
+        <v>398</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>398</v>
+      </c>
+      <c r="C7" t="s">
+        <v>398</v>
+      </c>
+      <c r="D7" t="s">
+        <v>410</v>
+      </c>
+      <c r="E7" t="s">
+        <v>411</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>398</v>
+      </c>
+      <c r="E8" t="s">
+        <v>123</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>398</v>
+      </c>
+      <c r="E9" t="s">
+        <v>123</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5367,4 +5739,319 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>368</v>
+      </c>
+      <c r="C2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>165</v>
+      </c>
+      <c r="F2" t="s">
+        <v>369</v>
+      </c>
+      <c r="G2" t="s">
+        <v>370</v>
+      </c>
+      <c r="H2" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C3" t="s">
+        <v>368</v>
+      </c>
+      <c r="D3" t="s">
+        <v>372</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>373</v>
+      </c>
+      <c r="G3" t="s">
+        <v>374</v>
+      </c>
+      <c r="H3" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" t="s">
+        <v>368</v>
+      </c>
+      <c r="C4" t="s">
+        <v>368</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>322</v>
+      </c>
+      <c r="F4" t="s">
+        <v>376</v>
+      </c>
+      <c r="G4" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>368</v>
+      </c>
+      <c r="C5" t="s">
+        <v>368</v>
+      </c>
+      <c r="D5" t="s">
+        <v>378</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>379</v>
+      </c>
+      <c r="G5" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>368</v>
+      </c>
+      <c r="C6" t="s">
+        <v>368</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" t="s">
+        <v>381</v>
+      </c>
+      <c r="G6" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" t="s">
+        <v>368</v>
+      </c>
+      <c r="C7" t="s">
+        <v>368</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>322</v>
+      </c>
+      <c r="F7" t="s">
+        <v>383</v>
+      </c>
+      <c r="G7" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" t="s">
+        <v>368</v>
+      </c>
+      <c r="C8" t="s">
+        <v>368</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
+        <v>385</v>
+      </c>
+      <c r="G8" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>368</v>
+      </c>
+      <c r="C9" t="s">
+        <v>368</v>
+      </c>
+      <c r="D9" t="s">
+        <v>91</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" t="s">
+        <v>387</v>
+      </c>
+      <c r="G9" t="s">
+        <v>388</v>
+      </c>
+      <c r="H9" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>368</v>
+      </c>
+      <c r="C10" t="s">
+        <v>368</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>390</v>
+      </c>
+      <c r="G10" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>368</v>
+      </c>
+      <c r="C11" t="s">
+        <v>368</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
+        <v>392</v>
+      </c>
+      <c r="F11" t="s">
+        <v>393</v>
+      </c>
+      <c r="G11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>368</v>
+      </c>
+      <c r="E12" t="s">
+        <v>123</v>
+      </c>
+      <c r="F12" t="s">
+        <v>395</v>
+      </c>
+      <c r="G12" t="s">
+        <v>127</v>
+      </c>
+      <c r="H12" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>368</v>
+      </c>
+      <c r="E13" t="s">
+        <v>123</v>
+      </c>
+      <c r="F13" t="s">
+        <v>396</v>
+      </c>
+      <c r="G13" t="s">
+        <v>397</v>
+      </c>
+      <c r="H13" t="s">
+        <v>206</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>